<commit_message>
feat: add workflow-based evaluation process
</commit_message>
<xml_diff>
--- a/data/model/cutting_stock_model/assumption_set.xlsx
+++ b/data/model/cutting_stock_model/assumption_set.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wang ngai wong\Desktop\Document\Research\Confidence Modeling\Code\Evaluation Agent\data\model\cutting stock model\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wang ngai wong\Desktop\Document\Research\Confidence Modeling\Code\Evaluation Agent\data\model\cutting_stock_model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C185001-F766-42D9-9F1D-F17F46DA0F65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0452D173-1F37-485E-9421-321116A8ADA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5325" yWindow="2025" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29295" yWindow="405" windowWidth="21600" windowHeight="12510" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Assumption" sheetId="1" r:id="rId1"/>
+    <sheet name="Model" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="52">
   <si>
     <t>ID</t>
   </si>
@@ -178,6 +179,9 @@
   </si>
   <si>
     <t>The optimization model is assumed to search within a reduced set of feasible cutting patterns to ensure tractable computation; in reality, potentially valuable cutting configurations may exist outside the explored solution space.</t>
+  </si>
+  <si>
+    <t>The model represents a manufacturing production planning system. It is used to determine production schedules and allocate products to production lines. The purpose of the model is to support production planning and scheduling decisions in a manufacturing environment.</t>
   </si>
 </sst>
 </file>
@@ -717,4 +721,19 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66DD6D80-3C26-4E57-ACE8-6552056FEF04}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>